<commit_message>
add new Cases and Check
</commit_message>
<xml_diff>
--- a/Check.xlsx
+++ b/Check.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diman\Desktop\Диплом\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC95157F-C90E-4349-99E7-73C37E572338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE7C26A9-5700-46D0-AA75-D7701DB9A6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="68">
   <si>
     <t>Группа проверок/модуль</t>
   </si>
@@ -218,6 +218,12 @@
   </si>
   <si>
     <t>Авторизация в приложении с невалидными логином и паролем (ввод символов)</t>
+  </si>
+  <si>
+    <t>Цитаты</t>
+  </si>
+  <si>
+    <t>Разворачивание/сворачивание цитат</t>
   </si>
 </sst>
 </file>
@@ -291,7 +297,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -395,12 +401,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -422,6 +443,20 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -641,7 +676,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.44140625" customWidth="1"/>
@@ -1168,16 +1203,35 @@
       </c>
     </row>
     <row r="57" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A57" s="8"/>
-      <c r="B57" s="6" t="s">
+      <c r="A57" s="12"/>
+      <c r="B57" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="C57" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="C57" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B58" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C58" s="17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="18"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
+    <mergeCell ref="A58:A59"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
     <mergeCell ref="A56:A57"/>
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A11"/>
@@ -1186,7 +1240,7 @@
     <mergeCell ref="A38:A55"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="C2:C57" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C58" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>